<commit_message>
Enhance economic proposal for charging box distribution
- Updated the economic calculation page with three models for distributing network fees among garage members, ensuring clarity on costs and responsibilities.
- Introduced detailed tables for each model, illustrating the financial implications for both active and inactive members.
- Added a warning box to address discrepancies in previous calculations and clarify assumptions regarding member participation.
- Revised text for improved readability and understanding of the proposed models and their impact on future connections.
</commit_message>
<xml_diff>
--- a/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
+++ b/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Hemma/laddboxar/kalkyl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24A77099-3971-4629-843C-4C401AB3446A}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{396058E9-C935-4315-926F-EC70C73F1047}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="8">
   <si>
     <t>TOT</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>Tänkt fördelning av ökad kostnad för förstärkt nät (63 A, trefas)</t>
+  </si>
+  <si>
+    <t>Jämn fördelning av ökad kostnad för förstärkt nät (63 A, trefas)</t>
   </si>
 </sst>
 </file>
@@ -98,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -109,6 +112,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -124,6 +130,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>465353</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>180590</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Bildobjekt 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08B7C55E-1E73-6C59-64AF-6A0BA773EBF5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6562725" y="485775"/>
+          <a:ext cx="10971428" cy="3076190"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -423,207 +478,295 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E7D67D2-7783-4FF6-A919-4905669F0636}">
-  <dimension ref="D7:I30"/>
+  <dimension ref="D3:R31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
+    <row r="3" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <v>94</v>
+      </c>
+      <c r="G3">
+        <v>23</v>
+      </c>
+      <c r="H3">
+        <f>F3*G3</f>
+        <v>2162</v>
+      </c>
+      <c r="I3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="F7">
+      <c r="F7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="E8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2">
         <v>94</v>
       </c>
-      <c r="G7">
-        <v>23</v>
-      </c>
-      <c r="H7">
-        <f>F7*G7</f>
+      <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="H8" s="2">
+        <f>F8*G8</f>
+        <v>564</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="E9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F9">
+        <v>94</v>
+      </c>
+      <c r="G9">
+        <v>17</v>
+      </c>
+      <c r="H9" s="2">
+        <f>F9*G9</f>
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="E10" s="4"/>
+      <c r="H10" s="5">
+        <f>SUM(H8:H9)</f>
         <v>2162</v>
       </c>
-      <c r="I7" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="F9">
-        <v>200</v>
-      </c>
-      <c r="G9">
-        <v>6</v>
-      </c>
-      <c r="H9">
-        <f>F9*G9</f>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="F10">
-        <v>57</v>
-      </c>
-      <c r="G10">
-        <v>17</v>
-      </c>
-      <c r="H10">
-        <f>F10*G10</f>
-        <v>969</v>
-      </c>
     </row>
     <row r="11" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="H11" s="1">
-        <f>SUM(H9:H10)</f>
-        <v>2169</v>
-      </c>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="H12" s="1"/>
+      <c r="H12" s="5"/>
     </row>
     <row r="13" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D13" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="F14" s="3" t="s">
+      <c r="D14" s="1"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="F15" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H15" s="6" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="E15" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F15" s="2">
-        <v>218.66666666666654</v>
-      </c>
-      <c r="G15">
-        <v>6</v>
-      </c>
-      <c r="H15">
-        <f>F15*G15</f>
-        <v>1311.9999999999993</v>
       </c>
     </row>
     <row r="16" spans="4:9" x14ac:dyDescent="0.25">
       <c r="E16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="2">
+        <v>218.66666666666654</v>
+      </c>
+      <c r="G16">
+        <v>6</v>
+      </c>
+      <c r="H16" s="2">
+        <f>F16*G16</f>
+        <v>1311.9999999999993</v>
+      </c>
+    </row>
+    <row r="17" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E17" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <v>50</v>
       </c>
-      <c r="G16">
+      <c r="G17">
         <v>17</v>
       </c>
-      <c r="H16">
-        <f>F16*G16</f>
+      <c r="H17" s="2">
+        <f>F17*G17</f>
         <v>850</v>
       </c>
     </row>
-    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E17" s="4"/>
-      <c r="H17" s="1">
-        <f>SUM(H15:H16)</f>
+    <row r="18" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E18" s="4"/>
+      <c r="H18" s="5">
+        <f>SUM(H16:H17)</f>
         <v>2161.9999999999991</v>
       </c>
     </row>
-    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F21" s="3" t="s">
+    <row r="19" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="F22" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H22" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E22" s="4" t="s">
+      <c r="P22" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E23" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F23" s="2">
         <v>187.42857142857144</v>
       </c>
-      <c r="G22">
+      <c r="G23">
         <v>7</v>
-      </c>
-      <c r="H22" s="2">
-        <f>F22*G22</f>
-        <v>1312</v>
-      </c>
-    </row>
-    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E23" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F23">
-        <v>50</v>
-      </c>
-      <c r="G23">
-        <v>17</v>
       </c>
       <c r="H23" s="2">
         <f>F23*G23</f>
+        <v>1312</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="P23" s="2">
+        <v>94</v>
+      </c>
+      <c r="Q23">
+        <v>6</v>
+      </c>
+      <c r="R23">
+        <f>P23*Q23</f>
+        <v>564</v>
+      </c>
+    </row>
+    <row r="24" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24">
+        <v>50</v>
+      </c>
+      <c r="G24">
+        <v>17</v>
+      </c>
+      <c r="H24" s="2">
+        <f>F24*G24</f>
         <v>850</v>
       </c>
-    </row>
-    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E24" s="4"/>
-      <c r="H24" s="5">
-        <f>SUM(H22:H23)</f>
+      <c r="O24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P24">
+        <v>94</v>
+      </c>
+      <c r="Q24">
+        <v>17</v>
+      </c>
+      <c r="R24">
+        <f>P24*Q24</f>
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="25" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E25" s="4"/>
+      <c r="H25" s="5">
+        <f>SUM(H23:H24)</f>
         <v>2162</v>
       </c>
-    </row>
-    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="F27" s="3" t="s">
+      <c r="O25" s="4"/>
+      <c r="R25" s="1">
+        <f>SUM(R23:R24)</f>
+        <v>2162</v>
+      </c>
+    </row>
+    <row r="26" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="F28" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H28" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E28" s="4" t="s">
+    <row r="29" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E29" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F29" s="2">
         <v>164</v>
       </c>
-      <c r="G28">
+      <c r="G29">
         <v>8</v>
-      </c>
-      <c r="H28" s="2">
-        <f>F28*G28</f>
-        <v>1312</v>
-      </c>
-    </row>
-    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E29" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F29">
-        <v>50</v>
-      </c>
-      <c r="G29">
-        <v>17</v>
       </c>
       <c r="H29" s="2">
         <f>F29*G29</f>
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="30" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E30" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F30">
+        <v>50</v>
+      </c>
+      <c r="G30">
+        <v>17</v>
+      </c>
+      <c r="H30" s="2">
+        <f>F30*G30</f>
         <v>850</v>
       </c>
     </row>
-    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E30" s="4"/>
-      <c r="H30" s="5">
-        <f>SUM(H28:H29)</f>
+    <row r="31" spans="5:18" x14ac:dyDescent="0.25">
+      <c r="E31" s="4"/>
+      <c r="H31" s="5">
+        <f>SUM(H29:H30)</f>
         <v>2162</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor proposal terminology for consistency across pages
- Updated references to "Vårt förslag" to "Förslag" in multiple HTML files for uniformity.
- Revised text in the proposal page to enhance clarity and readability, ensuring a consistent presentation of the proposal's implications.
- Adjusted the README to reflect the updated terminology for better alignment with the proposal content.
</commit_message>
<xml_diff>
--- a/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
+++ b/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Hemma/laddboxar/kalkyl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{396058E9-C935-4315-926F-EC70C73F1047}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E6A516F-3C04-4BF8-BC8B-E9597450B3A1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
   </bookViews>
@@ -609,6 +609,10 @@
     </row>
     <row r="18" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E18" s="4"/>
+      <c r="G18" s="1">
+        <f>SUM(G16:G17)</f>
+        <v>23</v>
+      </c>
       <c r="H18" s="5">
         <f>SUM(H16:H17)</f>
         <v>2161.9999999999991</v>
@@ -648,14 +652,14 @@
         <v>4</v>
       </c>
       <c r="F23" s="2">
-        <v>187.42857142857144</v>
+        <v>194.57142857142867</v>
       </c>
       <c r="G23">
         <v>7</v>
       </c>
       <c r="H23" s="2">
         <f>F23*G23</f>
-        <v>1312</v>
+        <v>1362.0000000000007</v>
       </c>
       <c r="O23" s="4" t="s">
         <v>4</v>
@@ -679,11 +683,11 @@
         <v>50</v>
       </c>
       <c r="G24">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H24" s="2">
         <f>F24*G24</f>
-        <v>850</v>
+        <v>800</v>
       </c>
       <c r="O24" s="4" t="s">
         <v>5</v>
@@ -701,9 +705,13 @@
     </row>
     <row r="25" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E25" s="4"/>
+      <c r="G25" s="1">
+        <f>SUM(G23:G24)</f>
+        <v>23</v>
+      </c>
       <c r="H25" s="5">
         <f>SUM(H23:H24)</f>
-        <v>2162</v>
+        <v>2162.0000000000009</v>
       </c>
       <c r="O25" s="4"/>
       <c r="R25" s="1">
@@ -733,14 +741,14 @@
         <v>4</v>
       </c>
       <c r="F29" s="2">
-        <v>164</v>
+        <v>176.5</v>
       </c>
       <c r="G29">
         <v>8</v>
       </c>
       <c r="H29" s="2">
         <f>F29*G29</f>
-        <v>1312</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="30" spans="5:18" x14ac:dyDescent="0.25">
@@ -751,15 +759,19 @@
         <v>50</v>
       </c>
       <c r="G30">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H30" s="2">
         <f>F30*G30</f>
-        <v>850</v>
+        <v>750</v>
       </c>
     </row>
     <row r="31" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E31" s="4"/>
+      <c r="G31" s="1">
+        <f>SUM(G29:G30)</f>
+        <v>23</v>
+      </c>
       <c r="H31" s="5">
         <f>SUM(H29:H30)</f>
         <v>2162</v>

</xml_diff>

<commit_message>
Enhance charging box proposal with new cost scenarios and clarifications
- Added a new section detailing the one-time costs associated with installing fewer or no charging boxes, including estimated costs and implications for members.
- Introduced tables comparing financial scenarios for members with and without charging boxes, highlighting the benefits of collective installation.
- Updated warning and information boxes to clarify assumptions and encourage confirmation of estimates with Laddboxkillarna.
- Refined existing content for improved clarity and consistency across the proposal page.
</commit_message>
<xml_diff>
--- a/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
+++ b/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Hemma/laddboxar/kalkyl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E6A516F-3C04-4BF8-BC8B-E9597450B3A1}"/>
+  <xr:revisionPtr revIDLastSave="162" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6373B313-4CCF-4649-BC39-EFEB83EE3C08}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
+    <sheet name="Blad2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="17">
   <si>
     <t>TOT</t>
   </si>
@@ -58,6 +59,33 @@
   </si>
   <si>
     <t>Jämn fördelning av ökad kostnad för förstärkt nät (63 A, trefas)</t>
+  </si>
+  <si>
+    <t>SUMMA:</t>
+  </si>
+  <si>
+    <t>per medlem</t>
+  </si>
+  <si>
+    <t>Med sex laddboxar</t>
+  </si>
+  <si>
+    <t>Utan Laddboxar</t>
+  </si>
+  <si>
+    <t>Alt A (med ladboxar)</t>
+  </si>
+  <si>
+    <t>Alt B (Ingen laddbox)</t>
+  </si>
+  <si>
+    <t>Kommentar</t>
+  </si>
+  <si>
+    <t>(8 000 kr i för själva  laddboxen)</t>
+  </si>
+  <si>
+    <t>Har tagit bort 6 000*6, för att inga laddboxar installeras</t>
   </si>
 </sst>
 </file>
@@ -81,12 +109,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -101,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -115,6 +149,23 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -170,6 +221,55 @@
         <a:xfrm>
           <a:off x="6562725" y="485775"/>
           <a:ext cx="10971428" cy="3076190"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>303634</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>75677</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Bildobjekt 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C183DC1-987B-537C-D883-9B16E95D8965}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1343025" y="466725"/>
+          <a:ext cx="9323809" cy="4180952"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -781,4 +881,234 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE2526F4-4C9B-4364-8A3A-3CB00EDA31E1}">
+  <dimension ref="N13:W36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="21" max="21" width="19.85546875" customWidth="1"/>
+    <col min="22" max="22" width="24.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="13" spans="20:22" x14ac:dyDescent="0.25">
+      <c r="T13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="U13" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="20:22" x14ac:dyDescent="0.25">
+      <c r="T14" s="2">
+        <v>208093</v>
+      </c>
+      <c r="U14" s="2">
+        <f>208093-6*6000</f>
+        <v>172093</v>
+      </c>
+      <c r="V14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="20:22" x14ac:dyDescent="0.25">
+      <c r="T15" s="2">
+        <v>-90000</v>
+      </c>
+      <c r="U15" s="2"/>
+    </row>
+    <row r="16" spans="20:22" x14ac:dyDescent="0.25">
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+    </row>
+    <row r="17" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+    </row>
+    <row r="18" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T18" s="2">
+        <v>35875</v>
+      </c>
+      <c r="U18" s="2">
+        <v>35875</v>
+      </c>
+    </row>
+    <row r="19" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+    </row>
+    <row r="20" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+    </row>
+    <row r="23" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="S23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="T23" s="5">
+        <f>SUM(T14:T18)</f>
+        <v>153968</v>
+      </c>
+      <c r="U23" s="5">
+        <f>SUM(U14:U18)</f>
+        <v>207968</v>
+      </c>
+    </row>
+    <row r="26" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="S26" s="4"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="5"/>
+    </row>
+    <row r="28" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="U28" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="V28" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="T29" s="8">
+        <v>6</v>
+      </c>
+      <c r="U29" s="12">
+        <f>8000+T23/23</f>
+        <v>14694.260869565216</v>
+      </c>
+      <c r="V29" s="12">
+        <f>T29*U29</f>
+        <v>88165.565217391297</v>
+      </c>
+      <c r="W29" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T30" s="8">
+        <v>17</v>
+      </c>
+      <c r="U30" s="12">
+        <v>3870.7314578005098</v>
+      </c>
+      <c r="V30" s="12">
+        <f>T30*U30</f>
+        <v>65802.434782608674</v>
+      </c>
+    </row>
+    <row r="31" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="11"/>
+      <c r="T31" s="7">
+        <f>SUM(T29:T30)</f>
+        <v>23</v>
+      </c>
+      <c r="U31" s="13">
+        <f>SUM(U29:U30)</f>
+        <v>18564.992327365726</v>
+      </c>
+      <c r="V31" s="13">
+        <f>SUM(V29:V30)</f>
+        <v>153967.99999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
+      <c r="T33" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="U33" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="V33" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="N34" s="2">
+        <f>8000+U35</f>
+        <v>17042.08695652174</v>
+      </c>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T34" s="8">
+        <v>6</v>
+      </c>
+      <c r="U34" s="12">
+        <f>U23/23</f>
+        <v>9042.0869565217399</v>
+      </c>
+      <c r="V34" s="12">
+        <f>T34*U34</f>
+        <v>54252.52173913044</v>
+      </c>
+    </row>
+    <row r="35" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T35" s="8">
+        <v>17</v>
+      </c>
+      <c r="U35" s="12">
+        <f>U23/23</f>
+        <v>9042.0869565217399</v>
+      </c>
+      <c r="V35" s="12">
+        <f>T35*U35</f>
+        <v>153715.47826086957</v>
+      </c>
+    </row>
+    <row r="36" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="11"/>
+      <c r="T36" s="7">
+        <f>SUM(T34:T35)</f>
+        <v>23</v>
+      </c>
+      <c r="U36" s="13">
+        <f>SUM(U34:U35)</f>
+        <v>18084.17391304348</v>
+      </c>
+      <c r="V36" s="13">
+        <f>SUM(V34:V35)</f>
+        <v>207968</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update economic calculations and offer analysis for charging boxes
- Revised cost breakdowns to include VAT calculations, clarifying that the total offer price is 208,093 kr excluding VAT, with the total including VAT now accurately reflected as 260,116 kr.
- Updated the net cost after the Ladda bilen-bidraget to 170,116 kr, ensuring clarity on the financial implications for members.
- Enhanced information boxes to explain the VAT treatment of the offer and the separate nature of the government grant, improving understanding of the overall costs.
- Adjusted tables and scenarios to reflect the new calculations, ensuring consistency across all relevant documents.
</commit_message>
<xml_diff>
--- a/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
+++ b/Hemma/laddboxar/kalkyl/egen_laddbox_kalkyl.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Hemma/laddboxar/kalkyl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6373B313-4CCF-4649-BC39-EFEB83EE3C08}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{F5D5A4B3-B6F8-4C1B-B128-73D814372602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58B973AD-5203-4494-92FD-033F554AD6C8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A09AED65-6D04-41FB-A934-B57BAB721136}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
     <sheet name="Blad2" sheetId="2" r:id="rId2"/>
+    <sheet name="Blad3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="18">
   <si>
     <t>TOT</t>
   </si>
@@ -86,13 +87,16 @@
   </si>
   <si>
     <t>Har tagit bort 6 000*6, för att inga laddboxar installeras</t>
+  </si>
+  <si>
+    <t>Med moms. Har tagit bort 6 000*6, för att inga laddboxar installeras</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,6 +107,21 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -135,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -166,6 +185,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -269,6 +296,55 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1343025" y="466725"/>
+          <a:ext cx="9323809" cy="4180952"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>541759</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>28052</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Bildobjekt 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6BCCAD9-98C2-420B-9B43-57699F426E17}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="971550" y="466725"/>
           <a:ext cx="9323809" cy="4180952"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -878,6 +954,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1108,6 +1185,239 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A673926-E294-4805-8D00-5BC123913720}">
+  <dimension ref="N13:W36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="21" max="21" width="25.42578125" customWidth="1"/>
+    <col min="22" max="22" width="24.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="13" spans="19:22" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="S13" s="16"/>
+      <c r="T13" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="U13" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="V13" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="19:22" x14ac:dyDescent="0.25">
+      <c r="T14" s="2">
+        <f>208093*1.25</f>
+        <v>260116.25</v>
+      </c>
+      <c r="U14" s="2">
+        <f>(208093-6*6000)*1.25</f>
+        <v>215116.25</v>
+      </c>
+      <c r="V14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="19:22" x14ac:dyDescent="0.25">
+      <c r="T15" s="2">
+        <v>-90000</v>
+      </c>
+      <c r="U15" s="2"/>
+    </row>
+    <row r="16" spans="19:22" x14ac:dyDescent="0.25">
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+    </row>
+    <row r="17" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+    </row>
+    <row r="18" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T18" s="2">
+        <v>35875</v>
+      </c>
+      <c r="U18" s="2">
+        <v>35875</v>
+      </c>
+    </row>
+    <row r="19" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+    </row>
+    <row r="20" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+    </row>
+    <row r="23" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="S23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="T23" s="5">
+        <f>SUM(T14:T18)</f>
+        <v>205991.25</v>
+      </c>
+      <c r="U23" s="5">
+        <f>SUM(U14:U18)</f>
+        <v>250991.25</v>
+      </c>
+    </row>
+    <row r="26" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="S26" s="4"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="5"/>
+    </row>
+    <row r="28" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="U28" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="V28" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="T29" s="8">
+        <v>6</v>
+      </c>
+      <c r="U29" s="12">
+        <f>8000+T23/23</f>
+        <v>16956.141304347824</v>
+      </c>
+      <c r="V29" s="12">
+        <f>T29*U29</f>
+        <v>101736.84782608695</v>
+      </c>
+      <c r="W29" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T30" s="8">
+        <v>17</v>
+      </c>
+      <c r="U30" s="12">
+        <v>6132.597186700772</v>
+      </c>
+      <c r="V30" s="12">
+        <f>T30*U30</f>
+        <v>104254.15217391313</v>
+      </c>
+    </row>
+    <row r="31" spans="17:23" x14ac:dyDescent="0.25">
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="11"/>
+      <c r="T31" s="7">
+        <f>SUM(T29:T30)</f>
+        <v>23</v>
+      </c>
+      <c r="U31" s="13">
+        <f>SUM(U29:U30)</f>
+        <v>23088.738491048596</v>
+      </c>
+      <c r="V31" s="13">
+        <f>SUM(V29:V30)</f>
+        <v>205991.00000000006</v>
+      </c>
+    </row>
+    <row r="33" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
+      <c r="T33" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="U33" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="V33" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="N34" s="2">
+        <f>8000+U35</f>
+        <v>18912.66304347826</v>
+      </c>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T34" s="8">
+        <v>6</v>
+      </c>
+      <c r="U34" s="12">
+        <f>U23/23</f>
+        <v>10912.66304347826</v>
+      </c>
+      <c r="V34" s="12">
+        <f>T34*U34</f>
+        <v>65475.97826086956</v>
+      </c>
+    </row>
+    <row r="35" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="T35" s="8">
+        <v>17</v>
+      </c>
+      <c r="U35" s="12">
+        <f>U23/23</f>
+        <v>10912.66304347826</v>
+      </c>
+      <c r="V35" s="12">
+        <f>T35*U35</f>
+        <v>185515.27173913043</v>
+      </c>
+    </row>
+    <row r="36" spans="14:22" x14ac:dyDescent="0.25">
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="11"/>
+      <c r="T36" s="7">
+        <f>SUM(T34:T35)</f>
+        <v>23</v>
+      </c>
+      <c r="U36" s="13">
+        <f>SUM(U34:U35)</f>
+        <v>21825.32608695652</v>
+      </c>
+      <c r="V36" s="13">
+        <f>SUM(V34:V35)</f>
+        <v>250991.25</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>